<commit_message>
Remove all colors from the topic 3 literature matrix
Plain black text on white with black borders; PMID and DOI are plain
text so no viewer shows them in color.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QgqFT5Fkzz2mf4ivKRGXX
</commit_message>
<xml_diff>
--- a/downloads/Literature_Matrix_Eating_Working_Copy_with_Summary.xlsx
+++ b/downloads/Literature_Matrix_Eating_Working_Copy_with_Summary.xlsx
@@ -136,7 +136,7 @@
     <t xml:space="preserve">Links</t>
   </si>
   <si>
-    <t xml:space="preserve">PMID cells open PubMed; DOI cells open the article.</t>
+    <t xml:space="preserve">Search the PMID on pubmed.ncbi.nlm.nih.gov, or put https://doi.org/ in front of the DOI, to open each article.</t>
   </si>
   <si>
     <t xml:space="preserve">Literature Matrix: Eating Patterns, Sleep Health, and Physiological Recovery Among Adult Wearable Users</t>
@@ -3248,7 +3248,7 @@
     <numFmt numFmtId="166" formatCode="0%"/>
     <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3274,23 +3274,19 @@
     <font>
       <b val="true"/>
       <sz val="14"/>
-      <color rgb="FF1E5631"/>
       <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
       <sz val="10"/>
-      <color rgb="FF555555"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -3308,57 +3304,16 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <u val="single"/>
-      <sz val="10"/>
-      <color rgb="FF1E5631"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF1E5631"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1E5631"/>
-        <bgColor rgb="FF274E13"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2E7D32"/>
-        <bgColor rgb="FF008000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1F8F1"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -3367,18 +3322,19 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
       <right style="thin">
         <color rgb="FFBFBFBF"/>
       </right>
-      <top style="thin">
-        <color rgb="FFBFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -3407,7 +3363,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3420,11 +3376,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3436,11 +3392,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3448,40 +3404,20 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -3492,7 +3428,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3508,11 +3444,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3525,73 +3461,11 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF2E7D32"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF1F8F1"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC8E6C9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF274E13"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1E5631"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <charset val="1"/>
-        <family val="0"/>
-        <b val="1"/>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC8E6C9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3602,7 +3476,7 @@
       <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
@@ -3616,7 +3490,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF1F8F1"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -3629,10 +3503,10 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFC8E6C9"/>
+      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -3644,16 +3518,16 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF555555"/>
+      <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF2E7D32"/>
+      <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF274E13"/>
+      <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF1E5631"/>
+      <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -3854,17 +3728,23 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -3899,10 +3779,10 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
@@ -3969,10 +3849,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="4"/>
+      <c r="B18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
@@ -3998,7 +3878,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>35</v>
       </c>
@@ -4053,11 +3933,69 @@
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
+      <c r="AA1" s="2"/>
+      <c r="AB1" s="2"/>
+      <c r="AC1" s="2"/>
+      <c r="AD1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>38</v>
       </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
@@ -4275,7 +4213,7 @@
       <c r="AB5" s="10" t="n">
         <v>38788519</v>
       </c>
-      <c r="AC5" s="11" t="s">
+      <c r="AC5" s="6" t="s">
         <v>86</v>
       </c>
       <c r="AD5" s="6" t="s">
@@ -4283,83 +4221,83 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="J6" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="K6" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="L6" s="13" t="s">
+      <c r="L6" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="M6" s="13" t="s">
+      <c r="M6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="N6" s="13" t="s">
+      <c r="N6" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="13" t="s">
+      <c r="O6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P6" s="13" t="s">
+      <c r="P6" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="Q6" s="13" t="s">
+      <c r="Q6" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="R6" s="13" t="s">
+      <c r="R6" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="S6" s="13" t="s">
+      <c r="S6" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="T6" s="12" t="str">
+      <c r="T6" s="9" t="str">
         <f aca="false">IF(OR(U6="Y",V6="Y",W6="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U6" s="12"/>
-      <c r="V6" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W6" s="12"/>
-      <c r="X6" s="12"/>
-      <c r="Y6" s="12"/>
-      <c r="Z6" s="12"/>
-      <c r="AA6" s="12"/>
-      <c r="AB6" s="14" t="n">
+      <c r="U6" s="9"/>
+      <c r="V6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W6" s="9"/>
+      <c r="X6" s="9"/>
+      <c r="Y6" s="9"/>
+      <c r="Z6" s="9"/>
+      <c r="AA6" s="9"/>
+      <c r="AB6" s="10" t="n">
         <v>42581816</v>
       </c>
-      <c r="AC6" s="15" t="s">
+      <c r="AC6" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="AD6" s="13" t="s">
+      <c r="AD6" s="6" t="s">
         <v>101</v>
       </c>
     </row>
@@ -4441,7 +4379,7 @@
       <c r="AB7" s="10" t="n">
         <v>34511160</v>
       </c>
-      <c r="AC7" s="11" t="s">
+      <c r="AC7" s="6" t="s">
         <v>116</v>
       </c>
       <c r="AD7" s="6" t="s">
@@ -4449,89 +4387,89 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="I8" s="16" t="n">
+      <c r="I8" s="11" t="n">
         <v>0.688</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="J8" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K8" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="L8" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="M8" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="N8" s="13" t="s">
+      <c r="N8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O8" s="13" t="s">
+      <c r="O8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="13" t="s">
+      <c r="P8" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="Q8" s="13" t="s">
+      <c r="Q8" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="R8" s="13" t="s">
+      <c r="R8" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="S8" s="13" t="s">
+      <c r="S8" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="T8" s="12" t="str">
+      <c r="T8" s="9" t="str">
         <f aca="false">IF(OR(U8="Y",V8="Y",W8="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V8" s="12"/>
-      <c r="W8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="X8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y8" s="12"/>
-      <c r="Z8" s="12"/>
-      <c r="AA8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB8" s="14" t="n">
+      <c r="U8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V8" s="9"/>
+      <c r="W8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y8" s="9"/>
+      <c r="Z8" s="9"/>
+      <c r="AA8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB8" s="10" t="n">
         <v>41305630</v>
       </c>
-      <c r="AC8" s="15" t="s">
+      <c r="AC8" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="AD8" s="13" t="s">
+      <c r="AD8" s="6" t="s">
         <v>132</v>
       </c>
     </row>
@@ -4560,7 +4498,7 @@
       <c r="H9" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="11" t="n">
         <v>0.5</v>
       </c>
       <c r="J9" s="6" t="s">
@@ -4611,7 +4549,7 @@
       <c r="AB9" s="10" t="n">
         <v>34017207</v>
       </c>
-      <c r="AC9" s="11" t="s">
+      <c r="AC9" s="6" t="s">
         <v>147</v>
       </c>
       <c r="AD9" s="6" t="s">
@@ -4619,87 +4557,87 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="I10" s="16" t="n">
+      <c r="I10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J10" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="K10" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="L10" s="13" t="s">
+      <c r="L10" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="M10" s="13" t="s">
+      <c r="M10" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="N10" s="13" t="s">
+      <c r="N10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O10" s="13" t="s">
+      <c r="O10" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="P10" s="13" t="s">
+      <c r="P10" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="Q10" s="13" t="s">
+      <c r="Q10" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="R10" s="13" t="s">
+      <c r="R10" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="S10" s="13" t="s">
+      <c r="S10" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="T10" s="12" t="str">
+      <c r="T10" s="9" t="str">
         <f aca="false">IF(OR(U10="Y",V10="Y",W10="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U10" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V10" s="12"/>
-      <c r="W10" s="12"/>
-      <c r="X10" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y10" s="12"/>
-      <c r="Z10" s="12"/>
-      <c r="AA10" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB10" s="14" t="n">
+      <c r="U10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V10" s="9"/>
+      <c r="W10" s="9"/>
+      <c r="X10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y10" s="9"/>
+      <c r="Z10" s="9"/>
+      <c r="AA10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB10" s="10" t="n">
         <v>41975458</v>
       </c>
-      <c r="AC10" s="15" t="s">
+      <c r="AC10" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="AD10" s="13" t="s">
+      <c r="AD10" s="6" t="s">
         <v>164</v>
       </c>
     </row>
@@ -4781,7 +4719,7 @@
       <c r="AB11" s="10" t="n">
         <v>41232466</v>
       </c>
-      <c r="AC11" s="11" t="s">
+      <c r="AC11" s="6" t="s">
         <v>175</v>
       </c>
       <c r="AD11" s="6" t="s">
@@ -4789,87 +4727,87 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="9" t="n">
         <v>2022</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="13" t="s">
+      <c r="J12" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="K12" s="13" t="s">
+      <c r="K12" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="L12" s="13" t="s">
+      <c r="L12" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="M12" s="13" t="s">
+      <c r="M12" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="N12" s="13" t="s">
+      <c r="N12" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="O12" s="13" t="s">
+      <c r="O12" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="P12" s="13" t="s">
+      <c r="P12" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="Q12" s="13" t="s">
+      <c r="Q12" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="R12" s="13" t="s">
+      <c r="R12" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="S12" s="13" t="s">
+      <c r="S12" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="T12" s="12" t="str">
+      <c r="T12" s="9" t="str">
         <f aca="false">IF(OR(U12="Y",V12="Y",W12="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U12" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V12" s="12"/>
-      <c r="W12" s="12"/>
-      <c r="X12" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y12" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z12" s="12"/>
-      <c r="AA12" s="12"/>
-      <c r="AB12" s="14" t="n">
+      <c r="U12" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V12" s="9"/>
+      <c r="W12" s="9"/>
+      <c r="X12" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y12" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z12" s="9"/>
+      <c r="AA12" s="9"/>
+      <c r="AB12" s="10" t="n">
         <v>35534102</v>
       </c>
-      <c r="AC12" s="15" t="s">
+      <c r="AC12" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="AD12" s="13" t="s">
+      <c r="AD12" s="6" t="s">
         <v>191</v>
       </c>
     </row>
@@ -4949,7 +4887,7 @@
       <c r="AB13" s="10" t="n">
         <v>37375582</v>
       </c>
-      <c r="AC13" s="11" t="s">
+      <c r="AC13" s="6" t="s">
         <v>203</v>
       </c>
       <c r="AD13" s="6" t="s">
@@ -4957,85 +4895,85 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="I14" s="12" t="s">
+      <c r="I14" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="13" t="s">
+      <c r="J14" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="K14" s="13" t="s">
+      <c r="K14" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="L14" s="13" t="s">
+      <c r="L14" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="M14" s="13" t="s">
+      <c r="M14" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="N14" s="13" t="s">
+      <c r="N14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O14" s="13" t="s">
+      <c r="O14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P14" s="13" t="s">
+      <c r="P14" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="Q14" s="13" t="s">
+      <c r="Q14" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="R14" s="13" t="s">
+      <c r="R14" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="S14" s="13" t="s">
+      <c r="S14" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="T14" s="12" t="str">
+      <c r="T14" s="9" t="str">
         <f aca="false">IF(OR(U14="Y",V14="Y",W14="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U14" s="12"/>
-      <c r="V14" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W14" s="12"/>
-      <c r="X14" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y14" s="12"/>
-      <c r="Z14" s="12"/>
-      <c r="AA14" s="12"/>
-      <c r="AB14" s="14" t="n">
+      <c r="U14" s="9"/>
+      <c r="V14" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W14" s="9"/>
+      <c r="X14" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y14" s="9"/>
+      <c r="Z14" s="9"/>
+      <c r="AA14" s="9"/>
+      <c r="AB14" s="10" t="n">
         <v>39144285</v>
       </c>
-      <c r="AC14" s="15" t="s">
+      <c r="AC14" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="AD14" s="13" t="s">
+      <c r="AD14" s="6" t="s">
         <v>217</v>
       </c>
     </row>
@@ -5115,7 +5053,7 @@
       <c r="AB15" s="10" t="n">
         <v>40498475</v>
       </c>
-      <c r="AC15" s="11" t="s">
+      <c r="AC15" s="6" t="s">
         <v>229</v>
       </c>
       <c r="AD15" s="6" t="s">
@@ -5123,85 +5061,85 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="13" t="s">
+      <c r="A16" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="F16" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="G16" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="H16" s="13" t="s">
+      <c r="H16" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="I16" s="12" t="s">
+      <c r="I16" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J16" s="13" t="s">
+      <c r="J16" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="K16" s="13" t="s">
+      <c r="K16" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="L16" s="13" t="s">
+      <c r="L16" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="M16" s="13" t="s">
+      <c r="M16" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="N16" s="13" t="s">
+      <c r="N16" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O16" s="13" t="s">
+      <c r="O16" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P16" s="13" t="s">
+      <c r="P16" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="Q16" s="13" t="s">
+      <c r="Q16" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="R16" s="13" t="s">
+      <c r="R16" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="S16" s="13" t="s">
+      <c r="S16" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="T16" s="12" t="str">
+      <c r="T16" s="9" t="str">
         <f aca="false">IF(OR(U16="Y",V16="Y",W16="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U16" s="12"/>
-      <c r="V16" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W16" s="12"/>
-      <c r="X16" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y16" s="12"/>
-      <c r="Z16" s="12"/>
-      <c r="AA16" s="12"/>
-      <c r="AB16" s="14" t="n">
+      <c r="U16" s="9"/>
+      <c r="V16" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W16" s="9"/>
+      <c r="X16" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y16" s="9"/>
+      <c r="Z16" s="9"/>
+      <c r="AA16" s="9"/>
+      <c r="AB16" s="10" t="n">
         <v>41202521</v>
       </c>
-      <c r="AC16" s="15" t="s">
+      <c r="AC16" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="AD16" s="13" t="s">
+      <c r="AD16" s="6" t="s">
         <v>242</v>
       </c>
     </row>
@@ -5281,7 +5219,7 @@
       <c r="AB17" s="10" t="n">
         <v>41208478</v>
       </c>
-      <c r="AC17" s="11" t="s">
+      <c r="AC17" s="6" t="s">
         <v>254</v>
       </c>
       <c r="AD17" s="6" t="s">
@@ -5289,85 +5227,85 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="9" t="n">
         <v>2023</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="I18" s="12" t="s">
+      <c r="I18" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J18" s="13" t="s">
+      <c r="J18" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="K18" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="L18" s="13" t="s">
+      <c r="L18" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="M18" s="13" t="s">
+      <c r="M18" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="N18" s="13" t="s">
+      <c r="N18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O18" s="13" t="s">
+      <c r="O18" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="P18" s="13" t="s">
+      <c r="P18" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="Q18" s="13" t="s">
+      <c r="Q18" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="R18" s="13" t="s">
+      <c r="R18" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="S18" s="13" t="s">
+      <c r="S18" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="T18" s="12" t="str">
+      <c r="T18" s="9" t="str">
         <f aca="false">IF(OR(U18="Y",V18="Y",W18="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U18" s="12"/>
-      <c r="V18" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W18" s="12"/>
-      <c r="X18" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y18" s="12"/>
-      <c r="Z18" s="12"/>
-      <c r="AA18" s="12"/>
-      <c r="AB18" s="14" t="n">
+      <c r="U18" s="9"/>
+      <c r="V18" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W18" s="9"/>
+      <c r="X18" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y18" s="9"/>
+      <c r="Z18" s="9"/>
+      <c r="AA18" s="9"/>
+      <c r="AB18" s="10" t="n">
         <v>37559551</v>
       </c>
-      <c r="AC18" s="15" t="s">
+      <c r="AC18" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="AD18" s="13" t="s">
+      <c r="AD18" s="6" t="s">
         <v>270</v>
       </c>
     </row>
@@ -5396,7 +5334,7 @@
       <c r="H19" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="I19" s="17" t="n">
+      <c r="I19" s="11" t="n">
         <v>0.92</v>
       </c>
       <c r="J19" s="6" t="s">
@@ -5447,7 +5385,7 @@
       <c r="AB19" s="10" t="n">
         <v>40241264</v>
       </c>
-      <c r="AC19" s="11" t="s">
+      <c r="AC19" s="6" t="s">
         <v>281</v>
       </c>
       <c r="AD19" s="6" t="s">
@@ -5455,87 +5393,87 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="F20" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="G20" s="13" t="s">
+      <c r="G20" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="H20" s="13" t="s">
+      <c r="H20" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="I20" s="16" t="n">
+      <c r="I20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J20" s="13" t="s">
+      <c r="J20" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="K20" s="13" t="s">
+      <c r="K20" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="L20" s="13" t="s">
+      <c r="L20" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="M20" s="13" t="s">
+      <c r="M20" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="N20" s="13" t="s">
+      <c r="N20" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O20" s="13" t="s">
+      <c r="O20" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="P20" s="13" t="s">
+      <c r="P20" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="Q20" s="13" t="s">
+      <c r="Q20" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="R20" s="13" t="s">
+      <c r="R20" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="S20" s="13" t="s">
+      <c r="S20" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="T20" s="12" t="str">
+      <c r="T20" s="9" t="str">
         <f aca="false">IF(OR(U20="Y",V20="Y",W20="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U20" s="12"/>
-      <c r="V20" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W20" s="12"/>
-      <c r="X20" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y20" s="12"/>
-      <c r="Z20" s="12"/>
-      <c r="AA20" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB20" s="14" t="n">
+      <c r="U20" s="9"/>
+      <c r="V20" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W20" s="9"/>
+      <c r="X20" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y20" s="9"/>
+      <c r="Z20" s="9"/>
+      <c r="AA20" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB20" s="10" t="n">
         <v>42272904</v>
       </c>
-      <c r="AC20" s="15" t="s">
+      <c r="AC20" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="AD20" s="13" t="s">
+      <c r="AD20" s="6" t="s">
         <v>296</v>
       </c>
     </row>
@@ -5615,7 +5553,7 @@
       <c r="AB21" s="10" t="n">
         <v>39458522</v>
       </c>
-      <c r="AC21" s="11" t="s">
+      <c r="AC21" s="6" t="s">
         <v>307</v>
       </c>
       <c r="AD21" s="6" t="s">
@@ -5623,85 +5561,85 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="n">
+      <c r="A22" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="G22" s="13" t="s">
+      <c r="G22" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="H22" s="13" t="s">
+      <c r="H22" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="I22" s="12" t="s">
+      <c r="I22" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J22" s="13" t="s">
+      <c r="J22" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="K22" s="13" t="s">
+      <c r="K22" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="L22" s="13" t="s">
+      <c r="L22" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="M22" s="13" t="s">
+      <c r="M22" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="N22" s="13" t="s">
+      <c r="N22" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O22" s="13" t="s">
+      <c r="O22" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="P22" s="13" t="s">
+      <c r="P22" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="Q22" s="13" t="s">
+      <c r="Q22" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="R22" s="13" t="s">
+      <c r="R22" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="S22" s="13" t="s">
+      <c r="S22" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="T22" s="12" t="str">
+      <c r="T22" s="9" t="str">
         <f aca="false">IF(OR(U22="Y",V22="Y",W22="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U22" s="12"/>
-      <c r="V22" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W22" s="12"/>
-      <c r="X22" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y22" s="12"/>
-      <c r="Z22" s="12"/>
-      <c r="AA22" s="12"/>
-      <c r="AB22" s="14" t="n">
+      <c r="U22" s="9"/>
+      <c r="V22" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W22" s="9"/>
+      <c r="X22" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y22" s="9"/>
+      <c r="Z22" s="9"/>
+      <c r="AA22" s="9"/>
+      <c r="AB22" s="10" t="n">
         <v>39182275</v>
       </c>
-      <c r="AC22" s="15" t="s">
+      <c r="AC22" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="AD22" s="13" t="s">
+      <c r="AD22" s="6" t="s">
         <v>323</v>
       </c>
     </row>
@@ -5783,7 +5721,7 @@
       <c r="AB23" s="10" t="n">
         <v>37083715</v>
       </c>
-      <c r="AC23" s="11" t="s">
+      <c r="AC23" s="6" t="s">
         <v>336</v>
       </c>
       <c r="AD23" s="6" t="s">
@@ -5791,87 +5729,87 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C24" s="9" t="n">
         <v>2023</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="F24" s="13" t="s">
+      <c r="F24" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="G24" s="13" t="s">
+      <c r="G24" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="H24" s="13" t="s">
+      <c r="H24" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="I24" s="16" t="n">
+      <c r="I24" s="11" t="n">
         <v>0.723076923076923</v>
       </c>
-      <c r="J24" s="13" t="s">
+      <c r="J24" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="K24" s="13" t="s">
+      <c r="K24" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="L24" s="13" t="s">
+      <c r="L24" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="M24" s="13" t="s">
+      <c r="M24" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="N24" s="13" t="s">
+      <c r="N24" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O24" s="13" t="s">
+      <c r="O24" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P24" s="13" t="s">
+      <c r="P24" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="Q24" s="13" t="s">
+      <c r="Q24" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="R24" s="13" t="s">
+      <c r="R24" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="S24" s="13" t="s">
+      <c r="S24" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="T24" s="12" t="str">
+      <c r="T24" s="9" t="str">
         <f aca="false">IF(OR(U24="Y",V24="Y",W24="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U24" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V24" s="12"/>
-      <c r="W24" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="X24" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y24" s="12"/>
-      <c r="Z24" s="12"/>
-      <c r="AA24" s="12"/>
-      <c r="AB24" s="14" t="n">
+      <c r="U24" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V24" s="9"/>
+      <c r="W24" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X24" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y24" s="9"/>
+      <c r="Z24" s="9"/>
+      <c r="AA24" s="9"/>
+      <c r="AB24" s="10" t="n">
         <v>37409467</v>
       </c>
-      <c r="AC24" s="15" t="s">
+      <c r="AC24" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AD24" s="13" t="s">
+      <c r="AD24" s="6" t="s">
         <v>350</v>
       </c>
     </row>
@@ -5900,7 +5838,7 @@
       <c r="H25" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="I25" s="17" t="n">
+      <c r="I25" s="11" t="n">
         <v>0.541666666666667</v>
       </c>
       <c r="J25" s="6" t="s">
@@ -5951,7 +5889,7 @@
       <c r="AB25" s="10" t="n">
         <v>37562755</v>
       </c>
-      <c r="AC25" s="11" t="s">
+      <c r="AC25" s="6" t="s">
         <v>362</v>
       </c>
       <c r="AD25" s="6" t="s">
@@ -5959,87 +5897,87 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="C26" s="12" t="n">
+      <c r="C26" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="F26" s="13" t="s">
+      <c r="F26" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="G26" s="13" t="s">
+      <c r="G26" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="I26" s="16" t="n">
+      <c r="I26" s="11" t="n">
         <v>0.671</v>
       </c>
-      <c r="J26" s="13" t="s">
+      <c r="J26" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="K26" s="13" t="s">
+      <c r="K26" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="L26" s="13" t="s">
+      <c r="L26" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="M26" s="13" t="s">
+      <c r="M26" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="N26" s="13" t="s">
+      <c r="N26" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O26" s="13" t="s">
+      <c r="O26" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P26" s="13" t="s">
+      <c r="P26" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="Q26" s="13" t="s">
+      <c r="Q26" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="R26" s="13" t="s">
+      <c r="R26" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="S26" s="13" t="s">
+      <c r="S26" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="T26" s="12" t="str">
+      <c r="T26" s="9" t="str">
         <f aca="false">IF(OR(U26="Y",V26="Y",W26="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U26" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V26" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W26" s="12"/>
-      <c r="X26" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y26" s="12"/>
-      <c r="Z26" s="12"/>
-      <c r="AA26" s="12"/>
-      <c r="AB26" s="14" t="n">
+      <c r="U26" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V26" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W26" s="9"/>
+      <c r="X26" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y26" s="9"/>
+      <c r="Z26" s="9"/>
+      <c r="AA26" s="9"/>
+      <c r="AB26" s="10" t="n">
         <v>40832902</v>
       </c>
-      <c r="AC26" s="15" t="s">
+      <c r="AC26" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="AD26" s="13" t="s">
+      <c r="AD26" s="6" t="s">
         <v>376</v>
       </c>
     </row>
@@ -6121,7 +6059,7 @@
       <c r="AB27" s="10" t="n">
         <v>41674465</v>
       </c>
-      <c r="AC27" s="11" t="s">
+      <c r="AC27" s="6" t="s">
         <v>390</v>
       </c>
       <c r="AD27" s="6" t="s">
@@ -6129,85 +6067,85 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="6" t="s">
         <v>392</v>
       </c>
-      <c r="C28" s="12" t="n">
+      <c r="C28" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="F28" s="13" t="s">
+      <c r="F28" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="G28" s="13" t="s">
+      <c r="G28" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="H28" s="13" t="s">
+      <c r="H28" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="I28" s="12" t="s">
+      <c r="I28" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J28" s="13" t="s">
+      <c r="J28" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="K28" s="13" t="s">
+      <c r="K28" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="L28" s="13" t="s">
+      <c r="L28" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="M28" s="13" t="s">
+      <c r="M28" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="N28" s="13" t="s">
+      <c r="N28" s="6" t="s">
         <v>399</v>
       </c>
-      <c r="O28" s="13" t="s">
+      <c r="O28" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P28" s="13" t="s">
+      <c r="P28" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="Q28" s="13" t="s">
+      <c r="Q28" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="R28" s="13" t="s">
+      <c r="R28" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="S28" s="13" t="s">
+      <c r="S28" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="T28" s="12" t="str">
+      <c r="T28" s="9" t="str">
         <f aca="false">IF(OR(U28="Y",V28="Y",W28="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U28" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V28" s="12"/>
-      <c r="W28" s="12"/>
-      <c r="X28" s="12"/>
-      <c r="Y28" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z28" s="12"/>
-      <c r="AA28" s="12"/>
-      <c r="AB28" s="14" t="n">
+      <c r="U28" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V28" s="9"/>
+      <c r="W28" s="9"/>
+      <c r="X28" s="9"/>
+      <c r="Y28" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z28" s="9"/>
+      <c r="AA28" s="9"/>
+      <c r="AB28" s="10" t="n">
         <v>40199860</v>
       </c>
-      <c r="AC28" s="15" t="s">
+      <c r="AC28" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="AD28" s="13" t="s">
+      <c r="AD28" s="6" t="s">
         <v>404</v>
       </c>
     </row>
@@ -6236,7 +6174,7 @@
       <c r="H29" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="I29" s="17" t="n">
+      <c r="I29" s="11" t="n">
         <v>0.368421052631579</v>
       </c>
       <c r="J29" s="6" t="s">
@@ -6285,7 +6223,7 @@
       <c r="AB29" s="10" t="n">
         <v>36095195</v>
       </c>
-      <c r="AC29" s="11" t="s">
+      <c r="AC29" s="6" t="s">
         <v>416</v>
       </c>
       <c r="AD29" s="6" t="s">
@@ -6293,85 +6231,85 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12" t="n">
+      <c r="A30" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C30" s="9" t="n">
         <v>2021</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="F30" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="G30" s="13" t="s">
+      <c r="G30" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="H30" s="13" t="s">
+      <c r="H30" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="I30" s="16" t="n">
+      <c r="I30" s="11" t="n">
         <v>0.48</v>
       </c>
-      <c r="J30" s="13" t="s">
+      <c r="J30" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="K30" s="13" t="s">
+      <c r="K30" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="L30" s="13" t="s">
+      <c r="L30" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="M30" s="13" t="s">
+      <c r="M30" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="N30" s="13" t="s">
+      <c r="N30" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="O30" s="13" t="s">
+      <c r="O30" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P30" s="13" t="s">
+      <c r="P30" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="Q30" s="13" t="s">
+      <c r="Q30" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="R30" s="13" t="s">
+      <c r="R30" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="S30" s="13" t="s">
+      <c r="S30" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="T30" s="12" t="str">
+      <c r="T30" s="9" t="str">
         <f aca="false">IF(OR(U30="Y",V30="Y",W30="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U30" s="12"/>
-      <c r="V30" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W30" s="12"/>
-      <c r="X30" s="12"/>
-      <c r="Y30" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z30" s="12"/>
-      <c r="AA30" s="12"/>
-      <c r="AB30" s="14" t="n">
+      <c r="U30" s="9"/>
+      <c r="V30" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W30" s="9"/>
+      <c r="X30" s="9"/>
+      <c r="Y30" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z30" s="9"/>
+      <c r="AA30" s="9"/>
+      <c r="AB30" s="10" t="n">
         <v>33859841</v>
       </c>
-      <c r="AC30" s="15" t="s">
+      <c r="AC30" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="AD30" s="13" t="s">
+      <c r="AD30" s="6" t="s">
         <v>431</v>
       </c>
     </row>
@@ -6400,7 +6338,7 @@
       <c r="H31" s="6" t="s">
         <v>436</v>
       </c>
-      <c r="I31" s="17" t="n">
+      <c r="I31" s="11" t="n">
         <v>0.66</v>
       </c>
       <c r="J31" s="6" t="s">
@@ -6455,7 +6393,7 @@
       <c r="AB31" s="10" t="n">
         <v>40797465</v>
       </c>
-      <c r="AC31" s="11" t="s">
+      <c r="AC31" s="6" t="s">
         <v>447</v>
       </c>
       <c r="AD31" s="6" t="s">
@@ -6463,85 +6401,85 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12" t="n">
+      <c r="A32" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="C32" s="12" t="n">
+      <c r="C32" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="E32" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="F32" s="13" t="s">
+      <c r="F32" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="G32" s="13" t="s">
+      <c r="G32" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="H32" s="13" t="s">
+      <c r="H32" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="I32" s="12" t="s">
+      <c r="I32" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J32" s="13" t="s">
+      <c r="J32" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="K32" s="13" t="s">
+      <c r="K32" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="L32" s="13" t="s">
+      <c r="L32" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M32" s="13" t="s">
+      <c r="M32" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="N32" s="13" t="s">
+      <c r="N32" s="6" t="s">
         <v>455</v>
       </c>
-      <c r="O32" s="13" t="s">
+      <c r="O32" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P32" s="13" t="s">
+      <c r="P32" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="Q32" s="13" t="s">
+      <c r="Q32" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="R32" s="13" t="s">
+      <c r="R32" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="S32" s="13" t="s">
+      <c r="S32" s="6" t="s">
         <v>459</v>
       </c>
-      <c r="T32" s="12" t="str">
+      <c r="T32" s="9" t="str">
         <f aca="false">IF(OR(U32="Y",V32="Y",W32="Y"),"Y","")</f>
         <v/>
       </c>
-      <c r="U32" s="12"/>
-      <c r="V32" s="12"/>
-      <c r="W32" s="12"/>
-      <c r="X32" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y32" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z32" s="12"/>
-      <c r="AA32" s="12"/>
-      <c r="AB32" s="14" t="n">
+      <c r="U32" s="9"/>
+      <c r="V32" s="9"/>
+      <c r="W32" s="9"/>
+      <c r="X32" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y32" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z32" s="9"/>
+      <c r="AA32" s="9"/>
+      <c r="AB32" s="10" t="n">
         <v>40895095</v>
       </c>
-      <c r="AC32" s="15" t="s">
+      <c r="AC32" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="AD32" s="13" t="s">
+      <c r="AD32" s="6" t="s">
         <v>461</v>
       </c>
     </row>
@@ -6623,7 +6561,7 @@
       <c r="AB33" s="10" t="n">
         <v>42189065</v>
       </c>
-      <c r="AC33" s="11" t="s">
+      <c r="AC33" s="6" t="s">
         <v>475</v>
       </c>
       <c r="AD33" s="6" t="s">
@@ -6631,83 +6569,83 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12" t="n">
+      <c r="A34" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="6" t="s">
         <v>477</v>
       </c>
-      <c r="C34" s="12" t="n">
+      <c r="C34" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="E34" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="F34" s="13" t="s">
+      <c r="F34" s="6" t="s">
         <v>479</v>
       </c>
-      <c r="G34" s="13" t="s">
+      <c r="G34" s="6" t="s">
         <v>480</v>
       </c>
-      <c r="H34" s="13" t="s">
+      <c r="H34" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="I34" s="16" t="n">
+      <c r="I34" s="11" t="n">
         <v>0.55</v>
       </c>
-      <c r="J34" s="13" t="s">
+      <c r="J34" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="K34" s="13" t="s">
+      <c r="K34" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="L34" s="13" t="s">
+      <c r="L34" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M34" s="13" t="s">
+      <c r="M34" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="N34" s="13" t="s">
+      <c r="N34" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O34" s="13" t="s">
+      <c r="O34" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="P34" s="13" t="s">
+      <c r="P34" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="Q34" s="13" t="s">
+      <c r="Q34" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="R34" s="13" t="s">
+      <c r="R34" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="S34" s="13" t="s">
+      <c r="S34" s="6" t="s">
         <v>459</v>
       </c>
-      <c r="T34" s="12" t="str">
+      <c r="T34" s="9" t="str">
         <f aca="false">IF(OR(U34="Y",V34="Y",W34="Y"),"Y","")</f>
         <v/>
       </c>
-      <c r="U34" s="12"/>
-      <c r="V34" s="12"/>
-      <c r="W34" s="12"/>
-      <c r="X34" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y34" s="12"/>
-      <c r="Z34" s="12"/>
-      <c r="AA34" s="12"/>
-      <c r="AB34" s="14" t="n">
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="10" t="n">
         <v>37738616</v>
       </c>
-      <c r="AC34" s="15" t="s">
+      <c r="AC34" s="6" t="s">
         <v>488</v>
       </c>
-      <c r="AD34" s="13" t="s">
+      <c r="AD34" s="6" t="s">
         <v>489</v>
       </c>
     </row>
@@ -6791,7 +6729,7 @@
       <c r="AB35" s="10" t="n">
         <v>41065723</v>
       </c>
-      <c r="AC35" s="11" t="s">
+      <c r="AC35" s="6" t="s">
         <v>503</v>
       </c>
       <c r="AD35" s="6" t="s">
@@ -6799,83 +6737,83 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12" t="n">
+      <c r="A36" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="C36" s="12" t="n">
+      <c r="C36" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="6" t="s">
         <v>506</v>
       </c>
-      <c r="E36" s="13" t="s">
+      <c r="E36" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="F36" s="13" t="s">
+      <c r="F36" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="G36" s="13" t="s">
+      <c r="G36" s="6" t="s">
         <v>507</v>
       </c>
-      <c r="H36" s="13" t="s">
+      <c r="H36" s="6" t="s">
         <v>508</v>
       </c>
-      <c r="I36" s="16" t="n">
+      <c r="I36" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J36" s="13" t="s">
+      <c r="J36" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="K36" s="13" t="s">
+      <c r="K36" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="L36" s="13" t="s">
+      <c r="L36" s="6" t="s">
         <v>509</v>
       </c>
-      <c r="M36" s="13" t="s">
+      <c r="M36" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="N36" s="13" t="s">
+      <c r="N36" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O36" s="13" t="s">
+      <c r="O36" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P36" s="13" t="s">
+      <c r="P36" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="Q36" s="13" t="s">
+      <c r="Q36" s="6" t="s">
         <v>511</v>
       </c>
-      <c r="R36" s="13" t="s">
+      <c r="R36" s="6" t="s">
         <v>512</v>
       </c>
-      <c r="S36" s="13" t="s">
+      <c r="S36" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="T36" s="12" t="str">
+      <c r="T36" s="9" t="str">
         <f aca="false">IF(OR(U36="Y",V36="Y",W36="Y"),"Y","")</f>
         <v/>
       </c>
-      <c r="U36" s="12"/>
-      <c r="V36" s="12"/>
-      <c r="W36" s="12"/>
-      <c r="X36" s="12"/>
-      <c r="Y36" s="12"/>
-      <c r="Z36" s="12"/>
-      <c r="AA36" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB36" s="14" t="n">
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB36" s="10" t="n">
         <v>39008822</v>
       </c>
-      <c r="AC36" s="15" t="s">
+      <c r="AC36" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="AD36" s="13" t="s">
+      <c r="AD36" s="6" t="s">
         <v>515</v>
       </c>
     </row>
@@ -6904,7 +6842,7 @@
       <c r="H37" s="6" t="s">
         <v>520</v>
       </c>
-      <c r="I37" s="17" t="n">
+      <c r="I37" s="11" t="n">
         <v>1</v>
       </c>
       <c r="J37" s="6" t="s">
@@ -6953,7 +6891,7 @@
       <c r="AB37" s="10" t="n">
         <v>41005066</v>
       </c>
-      <c r="AC37" s="11" t="s">
+      <c r="AC37" s="6" t="s">
         <v>527</v>
       </c>
       <c r="AD37" s="6" t="s">
@@ -6961,87 +6899,87 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="n">
+      <c r="A38" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B38" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C38" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="6" t="s">
         <v>530</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="6" t="s">
         <v>531</v>
       </c>
-      <c r="F38" s="13" t="s">
+      <c r="F38" s="6" t="s">
         <v>532</v>
       </c>
-      <c r="G38" s="13" t="s">
+      <c r="G38" s="6" t="s">
         <v>533</v>
       </c>
-      <c r="H38" s="13" t="s">
+      <c r="H38" s="6" t="s">
         <v>534</v>
       </c>
-      <c r="I38" s="16" t="n">
+      <c r="I38" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J38" s="13" t="s">
+      <c r="J38" s="6" t="s">
         <v>535</v>
       </c>
-      <c r="K38" s="13" t="s">
+      <c r="K38" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="L38" s="13" t="s">
+      <c r="L38" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M38" s="13" t="s">
+      <c r="M38" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="N38" s="13" t="s">
+      <c r="N38" s="6" t="s">
         <v>536</v>
       </c>
-      <c r="O38" s="13" t="s">
+      <c r="O38" s="6" t="s">
         <v>537</v>
       </c>
-      <c r="P38" s="13" t="s">
+      <c r="P38" s="6" t="s">
         <v>538</v>
       </c>
-      <c r="Q38" s="13" t="s">
+      <c r="Q38" s="6" t="s">
         <v>539</v>
       </c>
-      <c r="R38" s="13" t="s">
+      <c r="R38" s="6" t="s">
         <v>540</v>
       </c>
-      <c r="S38" s="13" t="s">
+      <c r="S38" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="T38" s="12" t="str">
+      <c r="T38" s="9" t="str">
         <f aca="false">IF(OR(U38="Y",V38="Y",W38="Y"),"Y","")</f>
         <v/>
       </c>
-      <c r="U38" s="12"/>
-      <c r="V38" s="12"/>
-      <c r="W38" s="12"/>
-      <c r="X38" s="12"/>
-      <c r="Y38" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z38" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA38" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB38" s="14" t="n">
+      <c r="U38" s="9"/>
+      <c r="V38" s="9"/>
+      <c r="W38" s="9"/>
+      <c r="X38" s="9"/>
+      <c r="Y38" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z38" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA38" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB38" s="10" t="n">
         <v>41545627</v>
       </c>
-      <c r="AC38" s="15" t="s">
+      <c r="AC38" s="6" t="s">
         <v>541</v>
       </c>
-      <c r="AD38" s="13" t="s">
+      <c r="AD38" s="6" t="s">
         <v>542</v>
       </c>
     </row>
@@ -7070,7 +7008,7 @@
       <c r="H39" s="6" t="s">
         <v>548</v>
       </c>
-      <c r="I39" s="17" t="n">
+      <c r="I39" s="11" t="n">
         <v>1</v>
       </c>
       <c r="J39" s="6" t="s">
@@ -7125,7 +7063,7 @@
       <c r="AB39" s="10" t="n">
         <v>35422659</v>
       </c>
-      <c r="AC39" s="11" t="s">
+      <c r="AC39" s="6" t="s">
         <v>557</v>
       </c>
       <c r="AD39" s="6" t="s">
@@ -7133,91 +7071,91 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12" t="n">
+      <c r="A40" s="9" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="6" t="s">
         <v>559</v>
       </c>
-      <c r="C40" s="12" t="n">
+      <c r="C40" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="D40" s="6" t="s">
         <v>560</v>
       </c>
-      <c r="E40" s="13" t="s">
+      <c r="E40" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="F40" s="13" t="s">
+      <c r="F40" s="6" t="s">
         <v>561</v>
       </c>
-      <c r="G40" s="13" t="s">
+      <c r="G40" s="6" t="s">
         <v>562</v>
       </c>
-      <c r="H40" s="13" t="s">
+      <c r="H40" s="6" t="s">
         <v>563</v>
       </c>
-      <c r="I40" s="16" t="n">
+      <c r="I40" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J40" s="13" t="s">
+      <c r="J40" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="K40" s="13" t="s">
+      <c r="K40" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="L40" s="13" t="s">
+      <c r="L40" s="6" t="s">
         <v>564</v>
       </c>
-      <c r="M40" s="13" t="s">
+      <c r="M40" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="N40" s="13" t="s">
+      <c r="N40" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O40" s="13" t="s">
+      <c r="O40" s="6" t="s">
         <v>566</v>
       </c>
-      <c r="P40" s="13" t="s">
+      <c r="P40" s="6" t="s">
         <v>567</v>
       </c>
-      <c r="Q40" s="13" t="s">
+      <c r="Q40" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="R40" s="13" t="s">
+      <c r="R40" s="6" t="s">
         <v>568</v>
       </c>
-      <c r="S40" s="13" t="s">
+      <c r="S40" s="6" t="s">
         <v>526</v>
       </c>
-      <c r="T40" s="12" t="str">
+      <c r="T40" s="9" t="str">
         <f aca="false">IF(OR(U40="Y",V40="Y",W40="Y"),"Y","")</f>
         <v>Y</v>
       </c>
-      <c r="U40" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V40" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="W40" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="X40" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y40" s="12"/>
-      <c r="Z40" s="12"/>
-      <c r="AA40" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB40" s="14" t="n">
+      <c r="U40" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V40" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W40" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X40" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y40" s="9"/>
+      <c r="Z40" s="9"/>
+      <c r="AA40" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB40" s="10" t="n">
         <v>42569180</v>
       </c>
-      <c r="AC40" s="15" t="s">
+      <c r="AC40" s="6" t="s">
         <v>569</v>
       </c>
-      <c r="AD40" s="13" t="s">
+      <c r="AD40" s="6" t="s">
         <v>570</v>
       </c>
     </row>
@@ -7297,7 +7235,7 @@
       <c r="AB41" s="10" t="n">
         <v>41596000</v>
       </c>
-      <c r="AC41" s="11" t="s">
+      <c r="AC41" s="6" t="s">
         <v>586</v>
       </c>
       <c r="AD41" s="6" t="s">
@@ -7305,85 +7243,85 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12" t="n">
+      <c r="A42" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="6" t="s">
         <v>588</v>
       </c>
-      <c r="C42" s="12" t="n">
+      <c r="C42" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="6" t="s">
         <v>589</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E42" s="6" t="s">
         <v>590</v>
       </c>
-      <c r="F42" s="13" t="s">
+      <c r="F42" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="G42" s="13" t="s">
+      <c r="G42" s="6" t="s">
         <v>591</v>
       </c>
-      <c r="H42" s="13" t="s">
+      <c r="H42" s="6" t="s">
         <v>592</v>
       </c>
-      <c r="I42" s="12" t="s">
+      <c r="I42" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J42" s="13" t="s">
+      <c r="J42" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="K42" s="13" t="s">
+      <c r="K42" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="L42" s="13" t="s">
+      <c r="L42" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M42" s="13" t="s">
+      <c r="M42" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="N42" s="13" t="s">
+      <c r="N42" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="O42" s="13" t="s">
+      <c r="O42" s="6" t="s">
         <v>595</v>
       </c>
-      <c r="P42" s="13" t="s">
+      <c r="P42" s="6" t="s">
         <v>596</v>
       </c>
-      <c r="Q42" s="13" t="s">
+      <c r="Q42" s="6" t="s">
         <v>597</v>
       </c>
-      <c r="R42" s="13" t="s">
+      <c r="R42" s="6" t="s">
         <v>598</v>
       </c>
-      <c r="S42" s="13" t="s">
+      <c r="S42" s="6" t="s">
         <v>599</v>
       </c>
-      <c r="T42" s="12" t="str">
+      <c r="T42" s="9" t="str">
         <f aca="false">IF(OR(U42="Y",V42="Y",W42="Y"),"Y","")</f>
         <v/>
       </c>
-      <c r="U42" s="12"/>
-      <c r="V42" s="12"/>
-      <c r="W42" s="12"/>
-      <c r="X42" s="12"/>
-      <c r="Y42" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z42" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA42" s="12"/>
-      <c r="AB42" s="14" t="n">
+      <c r="U42" s="9"/>
+      <c r="V42" s="9"/>
+      <c r="W42" s="9"/>
+      <c r="X42" s="9"/>
+      <c r="Y42" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z42" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA42" s="9"/>
+      <c r="AB42" s="10" t="n">
         <v>39788069</v>
       </c>
-      <c r="AC42" s="15" t="s">
+      <c r="AC42" s="6" t="s">
         <v>600</v>
       </c>
-      <c r="AD42" s="13" t="s">
+      <c r="AD42" s="6" t="s">
         <v>601</v>
       </c>
     </row>
@@ -7412,7 +7350,7 @@
       <c r="H43" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="I43" s="17" t="n">
+      <c r="I43" s="11" t="n">
         <v>0.490566037735849</v>
       </c>
       <c r="J43" s="6" t="s">
@@ -7465,7 +7403,7 @@
       <c r="AB43" s="10" t="n">
         <v>36016077</v>
       </c>
-      <c r="AC43" s="11" t="s">
+      <c r="AC43" s="6" t="s">
         <v>616</v>
       </c>
       <c r="AD43" s="6" t="s">
@@ -7473,85 +7411,85 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="n">
+      <c r="A44" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="13" t="s">
+      <c r="B44" s="6" t="s">
         <v>618</v>
       </c>
-      <c r="C44" s="12" t="n">
+      <c r="C44" s="9" t="n">
         <v>2021</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="6" t="s">
         <v>619</v>
       </c>
-      <c r="E44" s="13" t="s">
+      <c r="E44" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="F44" s="13" t="s">
+      <c r="F44" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="G44" s="13" t="s">
+      <c r="G44" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="H44" s="13" t="s">
+      <c r="H44" s="6" t="s">
         <v>620</v>
       </c>
-      <c r="I44" s="16" t="n">
+      <c r="I44" s="11" t="n">
         <v>0.647058823529412</v>
       </c>
-      <c r="J44" s="13" t="s">
+      <c r="J44" s="6" t="s">
         <v>621</v>
       </c>
-      <c r="K44" s="13" t="s">
+      <c r="K44" s="6" t="s">
         <v>609</v>
       </c>
-      <c r="L44" s="13" t="s">
+      <c r="L44" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M44" s="13" t="s">
+      <c r="M44" s="6" t="s">
         <v>622</v>
       </c>
-      <c r="N44" s="13" t="s">
+      <c r="N44" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O44" s="13" t="s">
+      <c r="O44" s="6" t="s">
         <v>623</v>
       </c>
-      <c r="P44" s="13" t="s">
+      <c r="P44" s="6" t="s">
         <v>624</v>
       </c>
-      <c r="Q44" s="13" t="s">
+      <c r="Q44" s="6" t="s">
         <v>625</v>
       </c>
-      <c r="R44" s="13" t="s">
+      <c r="R44" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="S44" s="13" t="s">
+      <c r="S44" s="6" t="s">
         <v>585</v>
       </c>
-      <c r="T44" s="12" t="str">
+      <c r="T44" s="9" t="str">
         <f aca="false">IF(OR(U44="Y",V44="Y",W44="Y"),"Y","")</f>
         <v/>
       </c>
-      <c r="U44" s="12"/>
-      <c r="V44" s="12"/>
-      <c r="W44" s="12"/>
-      <c r="X44" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y44" s="12"/>
-      <c r="Z44" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA44" s="12"/>
-      <c r="AB44" s="14" t="n">
+      <c r="U44" s="9"/>
+      <c r="V44" s="9"/>
+      <c r="W44" s="9"/>
+      <c r="X44" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y44" s="9"/>
+      <c r="Z44" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA44" s="9"/>
+      <c r="AB44" s="10" t="n">
         <v>33378539</v>
       </c>
-      <c r="AC44" s="15" t="s">
+      <c r="AC44" s="6" t="s">
         <v>627</v>
       </c>
-      <c r="AD44" s="13" t="s">
+      <c r="AD44" s="6" t="s">
         <v>628</v>
       </c>
     </row>
@@ -7580,7 +7518,7 @@
       <c r="H45" s="6" t="s">
         <v>632</v>
       </c>
-      <c r="I45" s="17" t="n">
+      <c r="I45" s="11" t="n">
         <v>0.461538461538462</v>
       </c>
       <c r="J45" s="6" t="s">
@@ -7631,7 +7569,7 @@
       <c r="AB45" s="10" t="n">
         <v>40834291</v>
       </c>
-      <c r="AC45" s="11" t="s">
+      <c r="AC45" s="6" t="s">
         <v>639</v>
       </c>
       <c r="AD45" s="6" t="s">
@@ -7639,85 +7577,85 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="12" t="n">
+      <c r="A46" s="9" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="13" t="s">
+      <c r="B46" s="6" t="s">
         <v>641</v>
       </c>
-      <c r="C46" s="12" t="n">
+      <c r="C46" s="9" t="n">
         <v>2021</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="6" t="s">
         <v>642</v>
       </c>
-      <c r="E46" s="13" t="s">
+      <c r="E46" s="6" t="s">
         <v>643</v>
       </c>
-      <c r="F46" s="13" t="s">
+      <c r="F46" s="6" t="s">
         <v>644</v>
       </c>
-      <c r="G46" s="13" t="s">
+      <c r="G46" s="6" t="s">
         <v>645</v>
       </c>
-      <c r="H46" s="13" t="s">
+      <c r="H46" s="6" t="s">
         <v>646</v>
       </c>
-      <c r="I46" s="16" t="n">
+      <c r="I46" s="11" t="n">
         <v>0.686868686868687</v>
       </c>
-      <c r="J46" s="13" t="s">
+      <c r="J46" s="6" t="s">
         <v>647</v>
       </c>
-      <c r="K46" s="13" t="s">
+      <c r="K46" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="L46" s="13" t="s">
+      <c r="L46" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M46" s="13" t="s">
+      <c r="M46" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="N46" s="13" t="s">
+      <c r="N46" s="6" t="s">
         <v>648</v>
       </c>
-      <c r="O46" s="13" t="s">
+      <c r="O46" s="6" t="s">
         <v>649</v>
       </c>
-      <c r="P46" s="13" t="s">
+      <c r="P46" s="6" t="s">
         <v>650</v>
       </c>
-      <c r="Q46" s="13" t="s">
+      <c r="Q46" s="6" t="s">
         <v>651</v>
       </c>
-      <c r="R46" s="13" t="s">
+      <c r="R46" s="6" t="s">
         <v>652</v>
       </c>
-      <c r="S46" s="13" t="s">
+      <c r="S46" s="6" t="s">
         <v>585</v>
       </c>
-      <c r="T46" s="12" t="str">
+      <c r="T46" s="9" t="str">
         <f aca="false">IF(OR(U46="Y",V46="Y",W46="Y"),"Y","")</f>
         <v/>
       </c>
-      <c r="U46" s="12"/>
-      <c r="V46" s="12"/>
-      <c r="W46" s="12"/>
-      <c r="X46" s="12"/>
-      <c r="Y46" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z46" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA46" s="12"/>
-      <c r="AB46" s="14" t="n">
+      <c r="U46" s="9"/>
+      <c r="V46" s="9"/>
+      <c r="W46" s="9"/>
+      <c r="X46" s="9"/>
+      <c r="Y46" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z46" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA46" s="9"/>
+      <c r="AB46" s="10" t="n">
         <v>33529156</v>
       </c>
-      <c r="AC46" s="15" t="s">
+      <c r="AC46" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="AD46" s="13" t="s">
+      <c r="AD46" s="6" t="s">
         <v>654</v>
       </c>
     </row>
@@ -7731,97 +7669,6 @@
     <mergeCell ref="T3:AA3"/>
     <mergeCell ref="AB3:AD3"/>
   </mergeCells>
-  <conditionalFormatting sqref="T5:AA46">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
-      <formula>"Y"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <hyperlinks>
-    <hyperlink ref="AB5" r:id="rId1" display="https://pubmed.ncbi.nlm.nih.gov/38788519/"/>
-    <hyperlink ref="AC5" r:id="rId2" display="10.1016/j.smrv.2024.101953"/>
-    <hyperlink ref="AB6" r:id="rId3" display="https://pubmed.ncbi.nlm.nih.gov/42581816/"/>
-    <hyperlink ref="AC6" r:id="rId4" display="10.1093/cvr/cvag169"/>
-    <hyperlink ref="AB7" r:id="rId5" display="https://pubmed.ncbi.nlm.nih.gov/34511160/"/>
-    <hyperlink ref="AC7" r:id="rId6" display="10.1017/S0007114521003597"/>
-    <hyperlink ref="AB8" r:id="rId7" display="https://pubmed.ncbi.nlm.nih.gov/41305630/"/>
-    <hyperlink ref="AC8" r:id="rId8" display="10.3390/nu17223580"/>
-    <hyperlink ref="AB9" r:id="rId9" display="https://pubmed.ncbi.nlm.nih.gov/34017207/"/>
-    <hyperlink ref="AC9" r:id="rId10" display="10.2147/NSS.S301113"/>
-    <hyperlink ref="AB10" r:id="rId11" display="https://pubmed.ncbi.nlm.nih.gov/41975458/"/>
-    <hyperlink ref="AC10" r:id="rId12" display="10.1186/s40101-026-00430-0"/>
-    <hyperlink ref="AB11" r:id="rId13" display="https://pubmed.ncbi.nlm.nih.gov/41232466/"/>
-    <hyperlink ref="AC11" r:id="rId14" display="10.1016/j.actpsy.2025.105900"/>
-    <hyperlink ref="AB12" r:id="rId15" display="https://pubmed.ncbi.nlm.nih.gov/35534102/"/>
-    <hyperlink ref="AC12" r:id="rId16" display="10.1016/j.jneb.2022.02.006"/>
-    <hyperlink ref="AB13" r:id="rId17" display="https://pubmed.ncbi.nlm.nih.gov/37375582/"/>
-    <hyperlink ref="AC13" r:id="rId18" display="10.3390/nu15122678"/>
-    <hyperlink ref="AB14" r:id="rId19" display="https://pubmed.ncbi.nlm.nih.gov/39144285/"/>
-    <hyperlink ref="AC14" r:id="rId20" display="10.3389/fnut.2024.1419811"/>
-    <hyperlink ref="AB15" r:id="rId21" display="https://pubmed.ncbi.nlm.nih.gov/40498475/"/>
-    <hyperlink ref="AC15" r:id="rId22" display="10.1093/nutrit/nuaf051"/>
-    <hyperlink ref="AB16" r:id="rId23" display="https://pubmed.ncbi.nlm.nih.gov/41202521/"/>
-    <hyperlink ref="AC16" r:id="rId24" display="10.1016/j.smrv.2025.102193"/>
-    <hyperlink ref="AB17" r:id="rId25" display="https://pubmed.ncbi.nlm.nih.gov/41208478/"/>
-    <hyperlink ref="AC17" r:id="rId26" display="10.1080/07420528.2025.2577859"/>
-    <hyperlink ref="AB18" r:id="rId27" display="https://pubmed.ncbi.nlm.nih.gov/37559551/"/>
-    <hyperlink ref="AC18" r:id="rId28" display="10.5664/jcsm.10754"/>
-    <hyperlink ref="AB19" r:id="rId29" display="https://pubmed.ncbi.nlm.nih.gov/40241264/"/>
-    <hyperlink ref="AC19" r:id="rId30" display="10.1093/sleep/zsaf089"/>
-    <hyperlink ref="AB20" r:id="rId31" display="https://pubmed.ncbi.nlm.nih.gov/42272904/"/>
-    <hyperlink ref="AC20" r:id="rId32" display="10.3389/fnut.2026.1823259"/>
-    <hyperlink ref="AB21" r:id="rId33" display="https://pubmed.ncbi.nlm.nih.gov/39458522/"/>
-    <hyperlink ref="AC21" r:id="rId34" display="10.3390/nu16203528"/>
-    <hyperlink ref="AB22" r:id="rId35" display="https://pubmed.ncbi.nlm.nih.gov/39182275/"/>
-    <hyperlink ref="AC22" r:id="rId36" display="10.1016/j.sleep.2024.08.012"/>
-    <hyperlink ref="AB23" r:id="rId37" display="https://pubmed.ncbi.nlm.nih.gov/37083715/"/>
-    <hyperlink ref="AC23" r:id="rId38" display="10.1093/sleep/zsad123"/>
-    <hyperlink ref="AB24" r:id="rId39" display="https://pubmed.ncbi.nlm.nih.gov/37409467/"/>
-    <hyperlink ref="AC24" r:id="rId40" display="10.5664/jcsm.10696"/>
-    <hyperlink ref="AB25" r:id="rId41" display="https://pubmed.ncbi.nlm.nih.gov/37562755/"/>
-    <hyperlink ref="AC25" r:id="rId42" display="10.1016/j.appet.2023.106998"/>
-    <hyperlink ref="AB26" r:id="rId43" display="https://pubmed.ncbi.nlm.nih.gov/40832902/"/>
-    <hyperlink ref="AC26" r:id="rId44" display="10.1093/sleep/zsaf247"/>
-    <hyperlink ref="AB27" r:id="rId45" display="https://pubmed.ncbi.nlm.nih.gov/41674465/"/>
-    <hyperlink ref="AC27" r:id="rId46" display="10.1161/ATVBAHA.125.323355"/>
-    <hyperlink ref="AB28" r:id="rId47" display="https://pubmed.ncbi.nlm.nih.gov/40199860/"/>
-    <hyperlink ref="AC28" r:id="rId48" display="10.1038/s41467-025-57846-y"/>
-    <hyperlink ref="AB29" r:id="rId49" display="https://pubmed.ncbi.nlm.nih.gov/36095195/"/>
-    <hyperlink ref="AC29" r:id="rId50" display="10.1073/pnas.2206348119"/>
-    <hyperlink ref="AB30" r:id="rId51" display="https://pubmed.ncbi.nlm.nih.gov/33859841/"/>
-    <hyperlink ref="AC30" r:id="rId52" display="10.1155/2021/6610455"/>
-    <hyperlink ref="AB31" r:id="rId53" display="https://pubmed.ncbi.nlm.nih.gov/40797465/"/>
-    <hyperlink ref="AC31" r:id="rId54" display="10.1097/MD.0000000000043800"/>
-    <hyperlink ref="AB32" r:id="rId55" display="https://pubmed.ncbi.nlm.nih.gov/40895095/"/>
-    <hyperlink ref="AC32" r:id="rId56" display="10.3389/fneur.2025.1556784"/>
-    <hyperlink ref="AB33" r:id="rId57" display="https://pubmed.ncbi.nlm.nih.gov/42189065/"/>
-    <hyperlink ref="AC33" r:id="rId58" display="10.1111/jce.70358"/>
-    <hyperlink ref="AB34" r:id="rId59" display="https://pubmed.ncbi.nlm.nih.gov/37738616/"/>
-    <hyperlink ref="AC34" r:id="rId60" display="10.1093/sleep/zsad253"/>
-    <hyperlink ref="AB35" r:id="rId61" display="https://pubmed.ncbi.nlm.nih.gov/41065723/"/>
-    <hyperlink ref="AC35" r:id="rId62" display="10.1093/sleep/zsaf318"/>
-    <hyperlink ref="AB36" r:id="rId63" display="https://pubmed.ncbi.nlm.nih.gov/39008822/"/>
-    <hyperlink ref="AC36" r:id="rId64" display="10.1093/nutrit/nuae093"/>
-    <hyperlink ref="AB37" r:id="rId65" display="https://pubmed.ncbi.nlm.nih.gov/41005066/"/>
-    <hyperlink ref="AC37" r:id="rId66" display="10.1016/j.appet.2025.108314"/>
-    <hyperlink ref="AB38" r:id="rId67" display="https://pubmed.ncbi.nlm.nih.gov/41545627/"/>
-    <hyperlink ref="AC38" r:id="rId68" display="10.1007/s40279-025-02388-y"/>
-    <hyperlink ref="AB39" r:id="rId69" display="https://pubmed.ncbi.nlm.nih.gov/35422659/"/>
-    <hyperlink ref="AC39" r:id="rId70" display="10.2147/ijwh.s341917"/>
-    <hyperlink ref="AB40" r:id="rId71" display="https://pubmed.ncbi.nlm.nih.gov/42569180/"/>
-    <hyperlink ref="AC40" r:id="rId72" display="10.3389/fnut.2026.1875559"/>
-    <hyperlink ref="AB41" r:id="rId73" display="https://pubmed.ncbi.nlm.nih.gov/41596000/"/>
-    <hyperlink ref="AC41" r:id="rId74" display="10.3390/bioengineering13010069"/>
-    <hyperlink ref="AB42" r:id="rId75" display="https://pubmed.ncbi.nlm.nih.gov/39788069/"/>
-    <hyperlink ref="AC42" r:id="rId76" display="10.1016/j.amjsurg.2024.116175"/>
-    <hyperlink ref="AB43" r:id="rId77" display="https://pubmed.ncbi.nlm.nih.gov/36016077/"/>
-    <hyperlink ref="AC43" r:id="rId78" display="10.3390/s22166317"/>
-    <hyperlink ref="AB44" r:id="rId79" display="https://pubmed.ncbi.nlm.nih.gov/33378539/"/>
-    <hyperlink ref="AC44" r:id="rId80" display="10.1093/sleep/zsaa291"/>
-    <hyperlink ref="AB45" r:id="rId81" display="https://pubmed.ncbi.nlm.nih.gov/40834291/"/>
-    <hyperlink ref="AC45" r:id="rId82" display="10.14814/phy2.70527"/>
-    <hyperlink ref="AB46" r:id="rId83" display="https://pubmed.ncbi.nlm.nih.gov/33529156/"/>
-    <hyperlink ref="AC46" r:id="rId84" display="10.2196/26107"/>
-  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="8" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -7829,7 +7676,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId85"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7849,642 +7696,681 @@
       <c r="A1" s="1" t="s">
         <v>655</v>
       </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>656</v>
       </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="12" t="s">
         <v>657</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="13" t="s">
         <v>658</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="13" t="s">
         <v>659</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="14" t="s">
         <v>660</v>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="15" t="n">
         <f aca="false">COUNTA('Literature Matrix'!$A$5:$A$46)</f>
         <v>42</v>
       </c>
-      <c r="C5" s="21"/>
+      <c r="C5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="17" t="s">
         <v>661</v>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$I$5:$I$46,"&gt;=0.5")</f>
         <v>17</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B6/$B$5)</f>
         <v>0.404761904761905</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="17" t="s">
         <v>662</v>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$I$5:$I$46,1)</f>
         <v>7</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B7/$B$5)</f>
         <v>0.166666666666667</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="17" t="s">
         <v>663</v>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$I$5:$I$46,"NR")</f>
         <v>13</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B8/$B$5)</f>
         <v>0.30952380952381</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="17" t="s">
         <v>664</v>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(AVERAGE('Literature Matrix'!$I$5:$I$46),0)</f>
         <v>0.732771269145123</v>
       </c>
-      <c r="C9" s="21"/>
+      <c r="C9" s="16"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="12" t="s">
         <v>665</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="13" t="s">
         <v>658</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="13" t="s">
         <v>659</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="17" t="s">
         <v>666</v>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$46,2021)</f>
         <v>4</v>
       </c>
-      <c r="C12" s="24" t="n">
+      <c r="C12" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B12/$B$5)</f>
         <v>0.0952380952380952</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="17" t="s">
         <v>667</v>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$46,2022)</f>
         <v>5</v>
       </c>
-      <c r="C13" s="24" t="n">
+      <c r="C13" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B13/$B$5)</f>
         <v>0.119047619047619</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="17" t="s">
         <v>668</v>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$46,2023)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="24" t="n">
+      <c r="C14" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B14/$B$5)</f>
         <v>0.119047619047619</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="17" t="s">
         <v>669</v>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$46,2024)</f>
         <v>5</v>
       </c>
-      <c r="C15" s="24" t="n">
+      <c r="C15" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B15/$B$5)</f>
         <v>0.119047619047619</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="17" t="s">
         <v>670</v>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$46,2025)</f>
         <v>12</v>
       </c>
-      <c r="C16" s="24" t="n">
+      <c r="C16" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B16/$B$5)</f>
         <v>0.285714285714286</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="17" t="s">
         <v>671</v>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$46,2026)</f>
         <v>11</v>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C17" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B17/$B$5)</f>
         <v>0.261904761904762</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="14" t="s">
         <v>672</v>
       </c>
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="15" t="n">
         <f aca="false">SUM(B12:B17)</f>
         <v>42</v>
       </c>
-      <c r="C18" s="24" t="n">
+      <c r="C18" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B18/$B$5)</f>
         <v>1</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="12" t="s">
         <v>673</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="13" t="s">
         <v>658</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="13" t="s">
         <v>659</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="B21" s="23" t="n">
+      <c r="B21" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$46,"Review")</f>
         <v>9</v>
       </c>
-      <c r="C21" s="24" t="n">
+      <c r="C21" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B21/$B$5)</f>
         <v>0.214285714285714</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="B22" s="23" t="n">
+      <c r="B22" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$46,"Cross-sectional")</f>
         <v>8</v>
       </c>
-      <c r="C22" s="24" t="n">
+      <c r="C22" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B22/$B$5)</f>
         <v>0.19047619047619</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="17" t="s">
         <v>316</v>
       </c>
-      <c r="B23" s="23" t="n">
+      <c r="B23" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$46,"Longitudinal / cohort")</f>
         <v>7</v>
       </c>
-      <c r="C23" s="24" t="n">
+      <c r="C23" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B23/$B$5)</f>
         <v>0.166666666666667</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="17" t="s">
         <v>329</v>
       </c>
-      <c r="B24" s="23" t="n">
+      <c r="B24" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$46,"Daily diary / repeated measures")</f>
         <v>1</v>
       </c>
-      <c r="C24" s="24" t="n">
+      <c r="C24" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B24/$B$5)</f>
         <v>0.0238095238095238</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="B25" s="23" t="n">
+      <c r="B25" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$46,"Randomized or controlled trial")</f>
         <v>11</v>
       </c>
-      <c r="C25" s="24" t="n">
+      <c r="C25" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B25/$B$5)</f>
         <v>0.261904761904762</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="17" t="s">
         <v>438</v>
       </c>
-      <c r="B26" s="23" t="n">
+      <c r="B26" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$46,"Single-arm / pre–post")</f>
         <v>3</v>
       </c>
-      <c r="C26" s="24" t="n">
+      <c r="C26" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B26/$B$5)</f>
         <v>0.0714285714285714</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="17" t="s">
         <v>609</v>
       </c>
-      <c r="B27" s="23" t="n">
+      <c r="B27" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$46,"Device validation")</f>
         <v>3</v>
       </c>
-      <c r="C27" s="24" t="n">
+      <c r="C27" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B27/$B$5)</f>
         <v>0.0714285714285714</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="14" t="s">
         <v>672</v>
       </c>
-      <c r="B28" s="20" t="n">
+      <c r="B28" s="15" t="n">
         <f aca="false">SUM(B21:B27)</f>
         <v>42</v>
       </c>
-      <c r="C28" s="24" t="n">
+      <c r="C28" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B28/$B$5)</f>
         <v>1</v>
       </c>
     </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+    </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="12" t="s">
         <v>674</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="13" t="s">
         <v>658</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="13" t="s">
         <v>659</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="23" t="n">
+      <c r="B31" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$T$5:$T$46,"Y")</f>
         <v>30</v>
       </c>
-      <c r="C31" s="24" t="n">
+      <c r="C31" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B31/$B$5)</f>
         <v>0.714285714285714</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="23" t="n">
+      <c r="B32" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$U$5:$U$46,"Y")</f>
         <v>15</v>
       </c>
-      <c r="C32" s="24" t="n">
+      <c r="C32" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B32/$B$5)</f>
         <v>0.357142857142857</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22" t="s">
+      <c r="A33" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B33" s="23" t="n">
+      <c r="B33" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$V$5:$V$46,"Y")</f>
         <v>18</v>
       </c>
-      <c r="C33" s="24" t="n">
+      <c r="C33" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B33/$B$5)</f>
         <v>0.428571428571429</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22" t="s">
+      <c r="A34" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="23" t="n">
+      <c r="B34" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$W$5:$W$46,"Y")</f>
         <v>7</v>
       </c>
-      <c r="C34" s="24" t="n">
+      <c r="C34" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B34/$B$5)</f>
         <v>0.166666666666667</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="B35" s="23" t="n">
+      <c r="B35" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$X$5:$X$46,"Y")</f>
         <v>30</v>
       </c>
-      <c r="C35" s="24" t="n">
+      <c r="C35" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B35/$B$5)</f>
         <v>0.714285714285714</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="23" t="n">
+      <c r="B36" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$Y$5:$Y$46,"Y")</f>
         <v>15</v>
       </c>
-      <c r="C36" s="24" t="n">
+      <c r="C36" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B36/$B$5)</f>
         <v>0.357142857142857</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B37" s="23" t="n">
+      <c r="B37" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$Z$5:$Z$46,"Y")</f>
         <v>10</v>
       </c>
-      <c r="C37" s="24" t="n">
+      <c r="C37" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B37/$B$5)</f>
         <v>0.238095238095238</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="23" t="n">
+      <c r="B38" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$AA$5:$AA$46,"Y")</f>
         <v>9</v>
       </c>
-      <c r="C38" s="24" t="n">
+      <c r="C38" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B38/$B$5)</f>
         <v>0.214285714285714</v>
       </c>
     </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+    </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
+      <c r="A40" s="12" t="s">
         <v>675</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="13" t="s">
         <v>658</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="13" t="s">
         <v>659</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="22" t="s">
+      <c r="A41" s="17" t="s">
         <v>676</v>
       </c>
-      <c r="B41" s="23" t="n">
+      <c r="B41" s="18" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$46,"Y",'Literature Matrix'!$X$5:$X$46,"Y")</f>
         <v>24</v>
       </c>
-      <c r="C41" s="24" t="n">
+      <c r="C41" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B41/$B$5)</f>
         <v>0.571428571428571</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="22" t="s">
+      <c r="A42" s="17" t="s">
         <v>677</v>
       </c>
-      <c r="B42" s="23" t="n">
+      <c r="B42" s="18" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$46,"Y",'Literature Matrix'!$Y$5:$Y$46,"Y")</f>
         <v>7</v>
       </c>
-      <c r="C42" s="24" t="n">
+      <c r="C42" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B42/$B$5)</f>
         <v>0.166666666666667</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="22" t="s">
+      <c r="A43" s="17" t="s">
         <v>678</v>
       </c>
-      <c r="B43" s="23" t="n">
+      <c r="B43" s="18" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$46,"Y",'Literature Matrix'!$X$5:$X$46,"Y",'Literature Matrix'!$Y$5:$Y$46,"Y")</f>
         <v>3</v>
       </c>
-      <c r="C43" s="24" t="n">
+      <c r="C43" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B43/$B$5)</f>
         <v>0.0714285714285714</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="22" t="s">
+      <c r="A44" s="17" t="s">
         <v>679</v>
       </c>
-      <c r="B44" s="23" t="n">
+      <c r="B44" s="18" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$46,"Y",'Literature Matrix'!$X$5:$X$46,"Y",'Literature Matrix'!$Y$5:$Y$46,"Y",'Literature Matrix'!$Z$5:$Z$46,"Y")</f>
         <v>2</v>
       </c>
-      <c r="C44" s="24" t="n">
+      <c r="C44" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B44/$B$5)</f>
         <v>0.0476190476190476</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="22" t="s">
+      <c r="A45" s="17" t="s">
         <v>680</v>
       </c>
-      <c r="B45" s="23" t="n">
+      <c r="B45" s="18" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$U$5:$U$46,"Y",'Literature Matrix'!$Y$5:$Y$46,"Y",'Literature Matrix'!$Z$5:$Z$46,"Y")</f>
         <v>0</v>
       </c>
-      <c r="C45" s="24" t="n">
+      <c r="C45" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B45/$B$5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="22" t="s">
+      <c r="A46" s="17" t="s">
         <v>681</v>
       </c>
-      <c r="B46" s="23" t="n">
+      <c r="B46" s="18" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$46,"Y",'Literature Matrix'!$Y$5:$Y$46,"Y",'Literature Matrix'!$AA$5:$AA$46,"Y")</f>
         <v>0</v>
       </c>
-      <c r="C46" s="24" t="n">
+      <c r="C46" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B46/$B$5)</f>
         <v>0</v>
       </c>
     </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+    </row>
     <row r="48" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="25" t="str">
+      <c r="A48" s="20" t="str">
         <f aca="false">"Gap: only "&amp;B44&amp;" of "&amp;B5&amp;" sources measured an eating pattern, sleep, and HRV/RHR with a consumer wearable; "&amp;IF(B45=0,"none",B45)&amp;" linked meal timing to HRV/RHR on a consumer wearable, and "&amp;IF(B46=0,"none",B46)&amp;" reported eating and HRV/RHR results for women."</f>
         <v>Gap: only 2 of 42 sources measured an eating pattern, sleep, and HRV/RHR with a consumer wearable; none linked meal timing to HRV/RHR on a consumer wearable, and none reported eating and HRV/RHR results for women.</v>
       </c>
-      <c r="B48" s="25"/>
-      <c r="C48" s="25"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
     </row>
     <row r="49" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="26" t="s">
+      <c r="A49" s="21" t="s">
         <v>682</v>
       </c>
-      <c r="B49" s="26"/>
-      <c r="C49" s="26"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="21"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="18" t="s">
+      <c r="A51" s="12" t="s">
         <v>683</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="B51" s="13" t="s">
         <v>658</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="C51" s="13" t="s">
         <v>659</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="22" t="s">
+      <c r="A52" s="17" t="s">
         <v>684</v>
       </c>
-      <c r="B52" s="23" t="n">
+      <c r="B52" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*Oura*")</f>
         <v>3</v>
       </c>
-      <c r="C52" s="24" t="n">
+      <c r="C52" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B52/$B$5)</f>
         <v>0.0714285714285714</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="22" t="s">
+      <c r="A53" s="17" t="s">
         <v>685</v>
       </c>
-      <c r="B53" s="23" t="n">
+      <c r="B53" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*Fitbit*")</f>
         <v>1</v>
       </c>
-      <c r="C53" s="24" t="n">
+      <c r="C53" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B53/$B$5)</f>
         <v>0.0238095238095238</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="22" t="s">
+      <c r="A54" s="17" t="s">
         <v>649</v>
       </c>
-      <c r="B54" s="23" t="n">
+      <c r="B54" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*Apple Watch*")</f>
         <v>2</v>
       </c>
-      <c r="C54" s="24" t="n">
+      <c r="C54" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B54/$B$5)</f>
         <v>0.0476190476190476</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="22" t="s">
+      <c r="A55" s="17" t="s">
         <v>686</v>
       </c>
-      <c r="B55" s="23" t="n">
+      <c r="B55" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*WHOOP*")</f>
         <v>3</v>
       </c>
-      <c r="C55" s="24" t="n">
+      <c r="C55" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B55/$B$5)</f>
         <v>0.0714285714285714</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="22" t="s">
+      <c r="A56" s="17" t="s">
         <v>687</v>
       </c>
-      <c r="B56" s="23" t="n">
+      <c r="B56" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*Garmin*")</f>
         <v>3</v>
       </c>
-      <c r="C56" s="24" t="n">
+      <c r="C56" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B56/$B$5)</f>
         <v>0.0714285714285714</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="22" t="s">
+      <c r="A57" s="17" t="s">
         <v>688</v>
       </c>
-      <c r="B57" s="23" t="n">
+      <c r="B57" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*Polar*")</f>
         <v>2</v>
       </c>
-      <c r="C57" s="24" t="n">
+      <c r="C57" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B57/$B$5)</f>
         <v>0.0476190476190476</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="22" t="s">
+      <c r="A58" s="17" t="s">
         <v>689</v>
       </c>
-      <c r="B58" s="23" t="n">
+      <c r="B58" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*Withings*")</f>
         <v>1</v>
       </c>
-      <c r="C58" s="24" t="n">
+      <c r="C58" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B58/$B$5)</f>
         <v>0.0238095238095238</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="22" t="s">
+      <c r="A59" s="17" t="s">
         <v>690</v>
       </c>
-      <c r="B59" s="23" t="n">
+      <c r="B59" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*Samsung*")</f>
         <v>1</v>
       </c>
-      <c r="C59" s="24" t="n">
+      <c r="C59" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B59/$B$5)</f>
         <v>0.0238095238095238</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="22" t="s">
+      <c r="A60" s="17" t="s">
         <v>691</v>
       </c>
-      <c r="B60" s="23" t="n">
+      <c r="B60" s="18" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$46,"*ctigraph*")</f>
         <v>5</v>
       </c>
-      <c r="C60" s="24" t="n">
+      <c r="C60" s="19" t="n">
         <f aca="false">IF($B$5=0,0,B60/$B$5)</f>
         <v>0.119047619047619</v>
       </c>

</xml_diff>